<commit_message>
ACDR2026: 10/9 opening speech review, participant list check, name tents update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011xF77D95cDW5CT1JUxj7vg
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_名札リスト_NameTents_案1009.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_名札リスト_NameTents_案1009.xlsx
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Based on the seating plan of 9 October. Line 1: country or organisation. Line 2: name (only where shown). Flag: Y = national flag on the tent.</t>
+          <t>Based on the seating plan and the participant list of 9 October. Line 1: country or organisation. Line 2: name (only where shown). Flag: Y = national flag on the tent.</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>名簿10/9: インドネシア（BNPB）は未登録【要確認】</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1720,7 +1724,11 @@
           <t>ADPC</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Mr Weerapon Sripongchai</t>
+        </is>
+      </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -1728,7 +1736,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>ADPC 4名予定（田中さん10/8）。2席で足りるか</t>
+          <t>名簿10/9: ADPCは2名（Perwaiz氏・Peeranan氏は不参加）</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1764,11 @@
           <t>ADPC</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Ms Apitsada Wetchakit</t>
+        </is>
+      </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -1862,7 +1874,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Mr KITAMOTO Masayuki</t>
+          <t>Mr KITAMOTO Masayuki, Board Member</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -1872,7 +1884,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>英文肩書【要確認】</t>
+          <t>名簿10/9: Board Member</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2148,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>内閣府随員。卓上プレートの要否【要確認】</t>
+          <t>内閣府随員。名簿10/9に内閣府は未登録。卓上プレートの要否【要確認】</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2332,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>TS発表者</t>
+          <t>TS発表者。名簿10/9の肩書はResearcher（コンセプトノートはSenior Researcher）【要確認】</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2748,11 @@
           <t>JICA</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr"/>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Mr NISHIKAWA Satoru, Senior Advisor</t>
+        </is>
+      </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -2744,7 +2760,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>氏名【要確認】</t>
+          <t>名簿10/9: JICA DRR Group</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2796,7 @@
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>KNFA（一般登録）の可能性【要確認】</t>
+          <t>名簿10/9: ROKはMOIS 4名（U字1・側面1・教室2）。KNFAのLee氏は一般参加で自由席</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ACDR2026: name tents to name/organisation format, check request draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011xF77D95cDW5CT1JUxj7vg
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_名札リスト_NameTents_案1009.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_名札リスト_NameTents_案1009.xlsx
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Based on the seating plan and the participant list of 9 October. Line 1: country or organisation. Line 2: name (only where shown). Flag: Y = national flag on the tent.</t>
+          <t>Based on the seating plan and the participant list of 9 October. Named tents: Line 1 = name, Line 2 = organisation (no job titles). Other tents: Line 1 = country or organisation only. Flag: Y = national flag on the tent.</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>Prof. MIURA Fusanori</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
           <t>ADRC</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Prof. MIURA Fusanori, Chairman</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
+          <t>Ms SAKURAI Noriko</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
           <t>JICA</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Ms SAKURAI Noriko, JICA DRR Policy Advisor to Fiji</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -1721,12 +1721,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
+          <t>Mr Weerapon Sripongchai</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
           <t>ADPC</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Mr Weerapon Sripongchai</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -1761,12 +1761,12 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
+          <t>Ms Apitsada Wetchakit</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
           <t>ADPC</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>Ms Apitsada Wetchakit</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -1833,12 +1833,12 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
+          <t>Mr MIYAKI Kazuhiro</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
           <t>ADRC</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>Mr MIYAKI Kazuhiro, Executive Director</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -1869,24 +1869,20 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
+          <t>Mr KITAMOTO Masayuki</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
           <t>ADRC</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>Mr KITAMOTO Masayuki, Board Member</t>
-        </is>
-      </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>名簿10/9: Board Member</t>
-        </is>
-      </c>
+      <c r="H45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -2205,12 +2201,12 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
+          <t>Mr TAKAHASHI Shinichi</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
           <t>City of Sendai</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>Mr TAKAHASHI Shinichi, Vice Mayor</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2277,14 +2273,14 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
+          <t>Ms MATSUO Naoko</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
           <t>JAXA</t>
         </is>
       </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>Ms MATSUO Naoko</t>
-        </is>
-      </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -2292,7 +2288,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>TS発表者。肩書【要確認】</t>
+          <t>TS発表者</t>
         </is>
       </c>
     </row>
@@ -2317,14 +2313,14 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
+          <t>Dr Yenni Vetrita</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
           <t>BRIN</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Dr Yenni Vetrita, Senior Researcher</t>
-        </is>
-      </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -2332,7 +2328,7 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>TS発表者。名簿10/9の肩書はResearcher（コンセプトノートはSenior Researcher）【要確認】</t>
+          <t>TS発表者。名簿10/9の肩書はResearcher。札は肩書なしなので影響なし</t>
         </is>
       </c>
     </row>
@@ -2357,14 +2353,14 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
+          <t>Ms Sirada Boonkongchuen</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
           <t>Google</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>Ms Sirada Boonkongchuen</t>
-        </is>
-      </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
           <t>N</t>
@@ -2372,7 +2368,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>RT発言・TS発表者（卓上マイク）。肩書【要確認】</t>
+          <t>RT発言・TS発表者（卓上マイク）</t>
         </is>
       </c>
     </row>
@@ -2397,12 +2393,12 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>YI-Lab, Nepal</t>
+          <t>Dr Pradip Khatiwada</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Dr Pradip Khatiwada, Founder and Executive Director</t>
+          <t>Youth Innovation Lab (YI-Lab), Nepal</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2673,12 +2669,12 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
+          <t>Ms UEDA Natsumi</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
           <t>JAXA</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>Ms UEDA Natsumi</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -2709,12 +2705,12 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
+          <t>Prof. ONO Yuichi</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
           <t>Tohoku University</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>Prof. ONO Yuichi</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -2745,12 +2741,12 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
+          <t>Mr NISHIKAWA Satoru</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
           <t>JICA</t>
-        </is>
-      </c>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
-          <t>Mr NISHIKAWA Satoru, Senior Advisor</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -2848,17 +2844,17 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Left table</t>
+          <t>Left table (Moderator)</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Moderator</t>
+          <t>LTC Chen Yong Kai</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>LTC Chen Yong Kai, SCDF</t>
+          <t>SCDF</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -2928,17 +2924,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Left table</t>
+          <t>Left table (Moderator)</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Moderator</t>
+          <t>LTC Chen Yong Kai</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>LTC Chen Yong Kai, SCDF</t>
+          <t>SCDF</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -2968,17 +2964,17 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Left table</t>
+          <t>Left table (Co-Chair)</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Co-Chair</t>
+          <t>Dr Mizan Bisri</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Dr Mizan Bisri, ADRC</t>
+          <t>ADRC</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -3013,12 +3009,12 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
+          <t>[TBC]</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
           <t>Uzbekistan</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3053,12 +3049,12 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
+          <t>Ms Sirada Boonkongchuen</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
           <t>Google</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
-          <t>Ms Sirada Boonkongchuen</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -3089,12 +3085,12 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
+          <t>Dr Yenni Vetrita</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
           <t>BRIN</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="inlineStr">
-        <is>
-          <t>Dr Yenni Vetrita</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -3125,12 +3121,12 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>YI-Lab, Nepal</t>
+          <t>Dr Pradip Khatiwada</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>Dr Pradip Khatiwada</t>
+          <t>Youth Innovation Lab (YI-Lab), Nepal</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -3161,12 +3157,12 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
+          <t>Ms MATSUO Naoko</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
           <t>JAXA</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>Ms MATSUO Naoko</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3197,12 +3193,12 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
+          <t>Mr NAKANE Toru</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
           <t>Cabinet Office of Japan</t>
-        </is>
-      </c>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
-          <t>Mr NAKANE Toru</t>
         </is>
       </c>
       <c r="G82" s="3" t="inlineStr">
@@ -3237,12 +3233,12 @@
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>WOTA</t>
+          <t>[TBC]</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>[TBC]</t>
+          <t>WOTA Corp.</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -3273,12 +3269,12 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Spectee</t>
+          <t>[TBC]</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>[TBC]</t>
+          <t>Spectee Inc.</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">

</xml_diff>

<commit_message>
ACDR2026: WOTA/Spectee seated behind Japan on stage, no name tents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011xF77D95cDW5CT1JUxj7vg
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/ACDR2026_名札リスト_NameTents_案1009.xlsx
+++ b/reports/acdr2026_staff_deployment/ACDR2026_名札リスト_NameTents_案1009.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3208,81 +3208,9 @@
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>右卓は6席。発表者8名なので日本の3名は教室型1列目から登壇する案【要確認】</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="3" t="n">
-        <v>79</v>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="inlineStr">
-        <is>
-          <t>Front: speakers table</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>Right table</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>WOTA Corp.</t>
-        </is>
-      </c>
-      <c r="G83" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H83" s="3" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="B84" s="3" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="C84" s="3" t="inlineStr">
-        <is>
-          <t>Front: speakers table</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>Right table</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="F84" s="3" t="inlineStr">
-        <is>
-          <t>Spectee Inc.</t>
-        </is>
-      </c>
-      <c r="G84" s="3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H84" s="3" t="inlineStr"/>
+          <t>右卓6席＝発表者6名（Uzbekistan〜内閣府）。WOTA・Spectee の2名はステージ上、日本の後ろに椅子のみ（名札なし）、発表は演台から（荒木田10/9）</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3390,7 +3318,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -3400,9 +3328,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>80</v>
-      </c>
-    </row>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>

</xml_diff>